<commit_message>
data: update Hob, KV
</commit_message>
<xml_diff>
--- a/xlsx/Hob.xlsx
+++ b/xlsx/Hob.xlsx
@@ -49131,7 +49131,7 @@
         <v>2803</v>
       </c>
     </row>
-    <row r="1132" s="2" customFormat="1" spans="1:12">
+    <row r="1132" s="2" customFormat="1" ht="138.85" spans="1:12">
       <c r="A1132" s="6">
         <v>20</v>
       </c>
@@ -49155,7 +49155,7 @@
         <v>1110</v>
       </c>
       <c r="I1132" s="6"/>
-      <c r="J1132" s="7" t="s">
+      <c r="J1132" s="14" t="s">
         <v>2790</v>
       </c>
       <c r="K1132" s="8" t="s">

</xml_diff>

<commit_message>
data: update Hob, MWV
</commit_message>
<xml_diff>
--- a/xlsx/Hob.xlsx
+++ b/xlsx/Hob.xlsx
@@ -9,12 +9,11 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView windowWidth="21925" windowHeight="9582"/>
+    <workbookView windowWidth="21942" windowHeight="9600"/>
   </bookViews>
   <sheets>
     <sheet name="Hob. " sheetId="2" r:id="rId1"/>
     <sheet name="Sheet1" sheetId="3" r:id="rId2"/>
-    <sheet name="Sheet2" sheetId="4" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Hob. '!$A$1:$J$1680</definedName>
@@ -57396,7 +57395,7 @@
     </row>
   </sheetData>
   <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:J1680" etc:filterBottomFollowUsedRange="0">
-    <sortState ref="A2:J1680">
+    <sortState ref="A1:J1680">
       <sortCondition ref="A1"/>
     </sortState>
     <extLst/>
@@ -57404,7 +57403,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
   <ignoredErrors>
-    <ignoredError sqref="F1:K1 D1 K2:K314" emptyCellReference="1"/>
+    <ignoredError sqref="K2:K314 D1 F1:K1" emptyCellReference="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -57759,15 +57758,4 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="8.61261261261261" defaultRowHeight="14.1"/>
-  <sheetData/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
-</worksheet>
 </file>
</xml_diff>